<commit_message>
Add Quants export (3) and fix R2 123 / MLMMJ product names
SRR2VIU123 maps to Verde Manzana per quant (3), not Azul Marino.
MLMMJDA66TS is MOTION LOOP MAFE DAMA per Odoo label.

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/SKU_ENTRADA_ALMACEN_completado.xlsx
+++ b/output/SKU_ENTRADA_ALMACEN_completado.xlsx
@@ -1628,7 +1628,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>MILA</t>
+          <t>MOTION LOOP MAFE DAMA</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -4055,12 +4055,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>quants:Quants__stock.quant___3__7680.xlsx</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>ok_quants_odoo</t>
         </is>
       </c>
     </row>
@@ -4173,7 +4173,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>R2 RUNNING 3,5" (Azul Marino, S)</t>
+          <t>R2 RUNNING 3,5" (Verde Manzana, S)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -4183,12 +4183,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>quants:Quants__stock.quant___3__7680.xlsx</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>ok_quants_odoo</t>
         </is>
       </c>
     </row>
@@ -4553,7 +4553,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>R2 RUNNING 3,5" (Azul Marino, M)</t>
+          <t>R2 RUNNING 3,5" (Verde Manzana, M)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -4563,12 +4563,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>quants:Quants__stock.quant___3__7680.xlsx</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>ok_quants_odoo</t>
         </is>
       </c>
     </row>
@@ -5146,7 +5146,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>R2 RUNNING 3,5" (Azul Marino, L)</t>
+          <t>R2 RUNNING 3,5" (Verde Manzana, L)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -5156,12 +5156,12 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>quants:Quants__stock.quant___3__7680.xlsx</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>ok_quants_odoo</t>
         </is>
       </c>
     </row>
@@ -5890,26 +5890,30 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>MILA</t>
+          <t>MOTION LOOP MAFE DAMA</t>
         </is>
       </c>
       <c r="C81" t="n">
         <v>3</v>
       </c>
-      <c r="D81" t="inlineStr"/>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>MOTION LOOP MAFE DAMA (Verde Militar, S)</t>
+        </is>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>MILMIDA66TS</t>
+          <t>MLMMJDA66TS</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>ok_catalog:alias_mila; global:MANUFACTURADO</t>
+          <t>odoo:known_label</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>ok_catalog:alias_mila</t>
+          <t>ok_odoo_known</t>
         </is>
       </c>
     </row>
@@ -6704,7 +6708,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>R2 RUNNING 3,5" (Azul Marino, XS)</t>
+          <t>R2 RUNNING 3,5" (Verde Manzana, XS)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -6714,12 +6718,12 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>quants:Quants__stock.quant___3__7680.xlsx</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>ok_quants_odoo</t>
         </is>
       </c>
     </row>
@@ -9754,12 +9758,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>quants:Quants__stock.quant___3__7680.xlsx</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>ok_quants_odoo</t>
         </is>
       </c>
     </row>
@@ -9779,7 +9783,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>R2 RUNNING 3,5" (Azul Marino, S)</t>
+          <t>R2 RUNNING 3,5" (Verde Manzana, S)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -9789,12 +9793,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>quants:Quants__stock.quant___3__7680.xlsx</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>ok_quants_odoo</t>
         </is>
       </c>
     </row>
@@ -9849,7 +9853,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>R2 RUNNING 3,5" (Azul Marino, M)</t>
+          <t>R2 RUNNING 3,5" (Verde Manzana, M)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -9859,12 +9863,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>quants:Quants__stock.quant___3__7680.xlsx</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>ok_quants_odoo</t>
         </is>
       </c>
     </row>
@@ -9884,7 +9888,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>R2 RUNNING 3,5" (Azul Marino, L)</t>
+          <t>R2 RUNNING 3,5" (Verde Manzana, L)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -9894,12 +9898,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>quants:Quants__stock.quant___3__7680.xlsx</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>ok_quants_odoo</t>
         </is>
       </c>
     </row>
@@ -9954,7 +9958,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>R2 RUNNING 3,5" (Azul Marino, XS)</t>
+          <t>R2 RUNNING 3,5" (Verde Manzana, XS)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -9964,12 +9968,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>quants:Quants__stock.quant___3__7680.xlsx</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>ok_quants_odoo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Quants export (4) to confirm last R2 Running SKUs
SRR2VIU43TL/TM/TXS now ok_quants_odoo; no remaining ok_r2_inferred.

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/SKU_ENTRADA_ALMACEN_completado.xlsx
+++ b/output/SKU_ENTRADA_ALMACEN_completado.xlsx
@@ -6753,12 +6753,12 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>quants:Quants__stock.quant___4__e718.xlsx</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>ok_quants_odoo</t>
         </is>
       </c>
     </row>
@@ -6788,12 +6788,12 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>quants:Quants__stock.quant___4__e718.xlsx</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>ok_quants_odoo</t>
         </is>
       </c>
     </row>
@@ -6823,12 +6823,12 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>quants:Quants__stock.quant___4__e718.xlsx</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>ok_quants_odoo</t>
         </is>
       </c>
     </row>
@@ -10003,12 +10003,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>quants:Quants__stock.quant___4__e718.xlsx</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>ok_quants_odoo</t>
         </is>
       </c>
     </row>
@@ -10038,12 +10038,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>quants:Quants__stock.quant___4__e718.xlsx</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>ok_quants_odoo</t>
         </is>
       </c>
     </row>
@@ -10073,12 +10073,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>quants:Quants__stock.quant___4__e718.xlsx</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>ok_r2_inferred</t>
+          <t>ok_quants_odoo</t>
         </is>
       </c>
     </row>

</xml_diff>